<commit_message>
docs: reconcile WBS status, routing decisions and handoff gates (2026-10-22)
</commit_message>
<xml_diff>
--- a/plans/wbs/otter-shield-wbs-print-a3-2pages.xlsx
+++ b/plans/wbs/otter-shield-wbs-print-a3-2pages.xlsx
@@ -629,7 +629,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>계획 기간은 옅은 칸으로 표시. 실제 진행한 날짜 칸을 색칠하고, 완료 확인 후 E열도 색칠하세요. 날짜 변경은 원본 WBS에 반영.</x:v>
+        <x:v>목표 기간은 옅은 칸. 수행일은 직접 색칠. 완료는 해당 작업 범위 기준이며 기술 검토와 구분합니다.</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -725,7 +725,7 @@
         <x:v>마감</x:v>
       </x:c>
       <x:c r="E5" s="14" t="str">
-        <x:v>완료</x:v>
+        <x:v>상태</x:v>
       </x:c>
       <x:c r="F5" s="14" t="str">
         <x:v>19</x:v>
@@ -820,7 +820,7 @@
         <x:v>I01</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>한국 본사 AS-IS 도면</x:v>
+        <x:v>한국 본사 AS-IS 토폴로지 작성</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
         <x:v>M1 유용수</x:v>
@@ -866,7 +866,7 @@
         <x:v>I02</x:v>
       </x:c>
       <x:c r="B7" s="39" t="str">
-        <x:v>독일 본사 AS-IS 도면</x:v>
+        <x:v>독일 AS-IS 토폴로지 작성</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
         <x:v>M2 윤서영</x:v>
@@ -874,7 +874,9 @@
       <x:c r="D7" s="40" t="str">
         <x:v>10/21</x:v>
       </x:c>
-      <x:c r="E7" s="41" t="str"/>
+      <x:c r="E7" s="41" t="str">
+        <x:v>검토 중</x:v>
+      </x:c>
       <x:c r="F7" s="29"/>
       <x:c r="G7" s="31"/>
       <x:c r="H7" s="31"/>
@@ -910,7 +912,7 @@
         <x:v>I03</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>한국 서비스 AS-IS 도면</x:v>
+        <x:v>한국 서비스망 AS-IS 토폴로지 작성</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
         <x:v>M3 홍은서</x:v>
@@ -918,7 +920,9 @@
       <x:c r="D8" s="23" t="str">
         <x:v>10/21</x:v>
       </x:c>
-      <x:c r="E8" s="24" t="str"/>
+      <x:c r="E8" s="24" t="str">
+        <x:v>완료</x:v>
+      </x:c>
       <x:c r="F8" s="29"/>
       <x:c r="G8" s="31"/>
       <x:c r="H8" s="31"/>
@@ -954,7 +958,7 @@
         <x:v>I04</x:v>
       </x:c>
       <x:c r="B9" s="39" t="str">
-        <x:v>백업·DR AS-IS 도면</x:v>
+        <x:v>백업·DR망 AS-IS 토폴로지 작성</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
         <x:v>M4 박진혁</x:v>
@@ -1000,7 +1004,7 @@
         <x:v>I05</x:v>
       </x:c>
       <x:c r="B10" s="22" t="str">
-        <x:v>캐나다 AS-IS 도면</x:v>
+        <x:v>캐나다 AS-IS 토폴로지 작성</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1008,7 +1012,9 @@
       <x:c r="D10" s="23" t="str">
         <x:v>10/21</x:v>
       </x:c>
-      <x:c r="E10" s="24" t="str"/>
+      <x:c r="E10" s="24" t="str">
+        <x:v>완료</x:v>
+      </x:c>
       <x:c r="F10" s="29"/>
       <x:c r="G10" s="31"/>
       <x:c r="H10" s="31"/>
@@ -1044,7 +1050,7 @@
         <x:v>C6.1</x:v>
       </x:c>
       <x:c r="B11" s="39" t="str">
-        <x:v>주소·환경 판정·계획서 검토</x:v>
+        <x:v>IP·구축 환경 기술 검토·계획서 개정</x:v>
       </x:c>
       <x:c r="C11" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1052,7 +1058,9 @@
       <x:c r="D11" s="40" t="str">
         <x:v>10/23</x:v>
       </x:c>
-      <x:c r="E11" s="41" t="str"/>
+      <x:c r="E11" s="41" t="str">
+        <x:v>진행 중</x:v>
+      </x:c>
       <x:c r="F11" s="29"/>
       <x:c r="G11" s="29"/>
       <x:c r="H11" s="31"/>
@@ -1088,7 +1096,7 @@
         <x:v>C10.1</x:v>
       </x:c>
       <x:c r="B12" s="22" t="str">
-        <x:v>DB 규격·복구 목표 합의</x:v>
+        <x:v>DB 구성·복구 목표 협의</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
         <x:v>M4 박진혁</x:v>
@@ -1096,7 +1104,9 @@
       <x:c r="D12" s="23" t="str">
         <x:v>10/23</x:v>
       </x:c>
-      <x:c r="E12" s="24" t="str"/>
+      <x:c r="E12" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
@@ -1132,7 +1142,7 @@
         <x:v>C12.1</x:v>
       </x:c>
       <x:c r="B13" s="39" t="str">
-        <x:v>AWS 권한·예산·API 판정</x:v>
+        <x:v>AWS 권한·예산·API 연결 검토</x:v>
       </x:c>
       <x:c r="C13" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1140,7 +1150,9 @@
       <x:c r="D13" s="40" t="str">
         <x:v>10/23</x:v>
       </x:c>
-      <x:c r="E13" s="41" t="str"/>
+      <x:c r="E13" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F13" s="29"/>
       <x:c r="G13" s="29"/>
       <x:c r="H13" s="31"/>
@@ -1176,7 +1188,7 @@
         <x:v>D1</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>실행 규격·ERD·Class 설계</x:v>
+        <x:v>실행 환경 정의·ERD·클래스 설계</x:v>
       </x:c>
       <x:c r="C14" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1184,7 +1196,9 @@
       <x:c r="D14" s="23" t="str">
         <x:v>10/23</x:v>
       </x:c>
-      <x:c r="E14" s="24" t="str"/>
+      <x:c r="E14" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F14" s="29"/>
       <x:c r="G14" s="29"/>
       <x:c r="H14" s="31"/>
@@ -1220,7 +1234,7 @@
         <x:v>D2</x:v>
       </x:c>
       <x:c r="B15" s="39" t="str">
-        <x:v>한국·독일 공통 게시판</x:v>
+        <x:v>한국·독일 공통 게시판 개발</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1228,7 +1242,9 @@
       <x:c r="D15" s="40" t="str">
         <x:v>10/23</x:v>
       </x:c>
-      <x:c r="E15" s="41" t="str"/>
+      <x:c r="E15" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F15" s="29"/>
       <x:c r="G15" s="29"/>
       <x:c r="H15" s="29"/>
@@ -1264,7 +1280,7 @@
         <x:v>I14</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>한국 장비·기본 서비스</x:v>
+        <x:v>한국 본사 장비·기본 서비스 구성</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
         <x:v>M1 유용수</x:v>
@@ -1272,7 +1288,9 @@
       <x:c r="D16" s="23" t="str">
         <x:v>10/28</x:v>
       </x:c>
-      <x:c r="E16" s="24" t="str"/>
+      <x:c r="E16" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F16" s="29"/>
       <x:c r="G16" s="29"/>
       <x:c r="H16" s="31"/>
@@ -1308,7 +1326,7 @@
         <x:v>I19</x:v>
       </x:c>
       <x:c r="B17" s="39" t="str">
-        <x:v>독일 장비·기본 서비스</x:v>
+        <x:v>독일 장비·기본 서비스 구성</x:v>
       </x:c>
       <x:c r="C17" s="40" t="str">
         <x:v>M2 윤서영</x:v>
@@ -1316,7 +1334,9 @@
       <x:c r="D17" s="40" t="str">
         <x:v>10/28</x:v>
       </x:c>
-      <x:c r="E17" s="41" t="str"/>
+      <x:c r="E17" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F17" s="29"/>
       <x:c r="G17" s="29"/>
       <x:c r="H17" s="31"/>
@@ -1352,7 +1372,7 @@
         <x:v>I24</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>한국 웹·K8s·DB 기반</x:v>
+        <x:v>한국 웹·K8s·DB 환경 구축</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
         <x:v>M3 홍은서</x:v>
@@ -1360,7 +1380,9 @@
       <x:c r="D18" s="23" t="str">
         <x:v>10/28</x:v>
       </x:c>
-      <x:c r="E18" s="24" t="str"/>
+      <x:c r="E18" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F18" s="29"/>
       <x:c r="G18" s="29"/>
       <x:c r="H18" s="31"/>
@@ -1396,7 +1418,7 @@
         <x:v>I29</x:v>
       </x:c>
       <x:c r="B19" s="39" t="str">
-        <x:v>백업망·시험 파일 기반</x:v>
+        <x:v>백업망 구축·테스트 파일 준비</x:v>
       </x:c>
       <x:c r="C19" s="40" t="str">
         <x:v>M4 박진혁</x:v>
@@ -1404,7 +1426,9 @@
       <x:c r="D19" s="40" t="str">
         <x:v>10/28</x:v>
       </x:c>
-      <x:c r="E19" s="41" t="str"/>
+      <x:c r="E19" s="41" t="str">
+        <x:v>진행 중</x:v>
+      </x:c>
       <x:c r="F19" s="29"/>
       <x:c r="G19" s="29"/>
       <x:c r="H19" s="31"/>
@@ -1440,7 +1464,7 @@
         <x:v>I34</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>캐나다 장비·기본 통신</x:v>
+        <x:v>캐나다 장비 구성·기본 통신 검증</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1448,7 +1472,9 @@
       <x:c r="D20" s="23" t="str">
         <x:v>10/28</x:v>
       </x:c>
-      <x:c r="E20" s="24" t="str"/>
+      <x:c r="E20" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F20" s="29"/>
       <x:c r="G20" s="29"/>
       <x:c r="H20" s="31"/>
@@ -1484,7 +1510,7 @@
         <x:v>C7</x:v>
       </x:c>
       <x:c r="B21" s="39" t="str">
-        <x:v>VPN·5개 망 왕복 연결</x:v>
+        <x:v>망 간 라우팅·VPN 구성 및 검증</x:v>
       </x:c>
       <x:c r="C21" s="40" t="str">
         <x:v>M1 유용수</x:v>
@@ -1492,7 +1518,9 @@
       <x:c r="D21" s="40" t="str">
         <x:v>10/28</x:v>
       </x:c>
-      <x:c r="E21" s="41" t="str"/>
+      <x:c r="E21" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F21" s="29"/>
       <x:c r="G21" s="29"/>
       <x:c r="H21" s="29"/>
@@ -1528,7 +1556,7 @@
         <x:v>D3</x:v>
       </x:c>
       <x:c r="B22" s="22" t="str">
-        <x:v>OTT 로그인·목록·샘플 재생</x:v>
+        <x:v>OTT 로그인·목록·영상 재생 개발</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1536,7 +1564,9 @@
       <x:c r="D22" s="23" t="str">
         <x:v>10/28</x:v>
       </x:c>
-      <x:c r="E22" s="24" t="str"/>
+      <x:c r="E22" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F22" s="29"/>
       <x:c r="G22" s="29"/>
       <x:c r="H22" s="29"/>
@@ -1572,7 +1602,7 @@
         <x:v>C10.2</x:v>
       </x:c>
       <x:c r="B23" s="39" t="str">
-        <x:v>Replica·격리 복원 준비</x:v>
+        <x:v>복제 DB·격리 복원 환경 준비</x:v>
       </x:c>
       <x:c r="C23" s="40" t="str">
         <x:v>M4 박진혁</x:v>
@@ -1580,7 +1610,9 @@
       <x:c r="D23" s="40" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E23" s="41" t="str"/>
+      <x:c r="E23" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F23" s="29"/>
       <x:c r="G23" s="29"/>
       <x:c r="H23" s="29"/>
@@ -1616,7 +1648,7 @@
         <x:v>C12.2</x:v>
       </x:c>
       <x:c r="B24" s="22" t="str">
-        <x:v>AWS 기반·재생성 명세</x:v>
+        <x:v>AWS 환경 구축·재구축 절차 작성</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1624,7 +1656,9 @@
       <x:c r="D24" s="23" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E24" s="24" t="str"/>
+      <x:c r="E24" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F24" s="29"/>
       <x:c r="G24" s="29"/>
       <x:c r="H24" s="29"/>
@@ -1660,7 +1694,7 @@
         <x:v>C6.2</x:v>
       </x:c>
       <x:c r="B25" s="39" t="str">
-        <x:v>공수·인계 준비 재점검</x:v>
+        <x:v>집중 업무 공수·배포 인계 점검</x:v>
       </x:c>
       <x:c r="C25" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1668,7 +1702,9 @@
       <x:c r="D25" s="40" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E25" s="41" t="str"/>
+      <x:c r="E25" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F25" s="29"/>
       <x:c r="G25" s="29"/>
       <x:c r="H25" s="29"/>
@@ -1704,7 +1740,7 @@
         <x:v>D4.1</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>한국 게시판 현지 배포</x:v>
+        <x:v>한국 게시판 서버 배포</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
         <x:v>M1 유용수</x:v>
@@ -1712,7 +1748,9 @@
       <x:c r="D26" s="23" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E26" s="24" t="str"/>
+      <x:c r="E26" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F26" s="29"/>
       <x:c r="G26" s="29"/>
       <x:c r="H26" s="29"/>
@@ -1748,7 +1786,7 @@
         <x:v>D4.2</x:v>
       </x:c>
       <x:c r="B27" s="39" t="str">
-        <x:v>독일 게시판 현지 배포</x:v>
+        <x:v>독일 게시판 서버 배포</x:v>
       </x:c>
       <x:c r="C27" s="40" t="str">
         <x:v>M2 윤서영</x:v>
@@ -1756,7 +1794,9 @@
       <x:c r="D27" s="40" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E27" s="41" t="str"/>
+      <x:c r="E27" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F27" s="29"/>
       <x:c r="G27" s="29"/>
       <x:c r="H27" s="29"/>
@@ -1792,7 +1832,7 @@
         <x:v>D4.3</x:v>
       </x:c>
       <x:c r="B28" s="22" t="str">
-        <x:v>한국 OTT 현지 배포</x:v>
+        <x:v>한국 OTT 서버 배포</x:v>
       </x:c>
       <x:c r="C28" s="23" t="str">
         <x:v>M3 홍은서</x:v>
@@ -1800,7 +1840,9 @@
       <x:c r="D28" s="23" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E28" s="24" t="str"/>
+      <x:c r="E28" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F28" s="29"/>
       <x:c r="G28" s="29"/>
       <x:c r="H28" s="29"/>
@@ -1844,7 +1886,9 @@
       <x:c r="D29" s="40" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E29" s="41" t="str"/>
+      <x:c r="E29" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F29" s="29"/>
       <x:c r="G29" s="29"/>
       <x:c r="H29" s="29"/>
@@ -1880,7 +1924,7 @@
         <x:v>D6.1</x:v>
       </x:c>
       <x:c r="B30" s="22" t="str">
-        <x:v>CI·이미지·배포 Git 준비</x:v>
+        <x:v>CI 구성·이미지·배포 저장소 준비</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -1888,7 +1932,9 @@
       <x:c r="D30" s="23" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E30" s="24" t="str"/>
+      <x:c r="E30" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F30" s="29"/>
       <x:c r="G30" s="29"/>
       <x:c r="H30" s="29"/>
@@ -1924,7 +1970,7 @@
         <x:v>I15</x:v>
       </x:c>
       <x:c r="B31" s="39" t="str">
-        <x:v>S01 공격 시험·원인 분석</x:v>
+        <x:v>S01 공격 재현·원인 분석</x:v>
       </x:c>
       <x:c r="C31" s="40" t="str">
         <x:v>M1 유용수</x:v>
@@ -1932,7 +1978,9 @@
       <x:c r="D31" s="40" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E31" s="41" t="str"/>
+      <x:c r="E31" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F31" s="29"/>
       <x:c r="G31" s="29"/>
       <x:c r="H31" s="29"/>
@@ -1968,7 +2016,7 @@
         <x:v>I20</x:v>
       </x:c>
       <x:c r="B32" s="22" t="str">
-        <x:v>S02 공격 시험·원인 분석</x:v>
+        <x:v>S02 공격 재현·원인 분석</x:v>
       </x:c>
       <x:c r="C32" s="23" t="str">
         <x:v>M2 윤서영</x:v>
@@ -1976,7 +2024,9 @@
       <x:c r="D32" s="23" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E32" s="24" t="str"/>
+      <x:c r="E32" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F32" s="29"/>
       <x:c r="G32" s="29"/>
       <x:c r="H32" s="29"/>
@@ -2012,7 +2062,7 @@
         <x:v>I30</x:v>
       </x:c>
       <x:c r="B33" s="39" t="str">
-        <x:v>S04 공격 시험·원인 분석</x:v>
+        <x:v>S04 공격 재현·원인 분석</x:v>
       </x:c>
       <x:c r="C33" s="40" t="str">
         <x:v>M4 박진혁</x:v>
@@ -2020,7 +2070,9 @@
       <x:c r="D33" s="40" t="str">
         <x:v>10/30</x:v>
       </x:c>
-      <x:c r="E33" s="41" t="str"/>
+      <x:c r="E33" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F33" s="29"/>
       <x:c r="G33" s="29"/>
       <x:c r="H33" s="29"/>
@@ -2056,7 +2108,7 @@
         <x:v>D5.2</x:v>
       </x:c>
       <x:c r="B34" s="22" t="str">
-        <x:v>Store AWS 첫 연결·배포</x:v>
+        <x:v>Store AWS 배포·서비스 연동</x:v>
       </x:c>
       <x:c r="C34" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -2064,7 +2116,9 @@
       <x:c r="D34" s="23" t="str">
         <x:v>10/31</x:v>
       </x:c>
-      <x:c r="E34" s="24" t="str"/>
+      <x:c r="E34" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F34" s="29"/>
       <x:c r="G34" s="29"/>
       <x:c r="H34" s="29"/>
@@ -2100,7 +2154,7 @@
         <x:v>D5.3</x:v>
       </x:c>
       <x:c r="B35" s="39" t="str">
-        <x:v>Store 잔여 문제·영향 판정</x:v>
+        <x:v>Store 오류 분석·일정 영향 검토</x:v>
       </x:c>
       <x:c r="C35" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -2108,7 +2162,9 @@
       <x:c r="D35" s="40" t="str">
         <x:v>11/02</x:v>
       </x:c>
-      <x:c r="E35" s="41" t="str"/>
+      <x:c r="E35" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F35" s="29"/>
       <x:c r="G35" s="29"/>
       <x:c r="H35" s="29"/>
@@ -2144,7 +2200,7 @@
         <x:v>I25</x:v>
       </x:c>
       <x:c r="B36" s="22" t="str">
-        <x:v>S03 공격 시험·원인 분석</x:v>
+        <x:v>S03 공격 재현·원인 분석</x:v>
       </x:c>
       <x:c r="C36" s="23" t="str">
         <x:v>M3 홍은서</x:v>
@@ -2152,7 +2208,9 @@
       <x:c r="D36" s="23" t="str">
         <x:v>11/02</x:v>
       </x:c>
-      <x:c r="E36" s="24" t="str"/>
+      <x:c r="E36" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F36" s="29"/>
       <x:c r="G36" s="29"/>
       <x:c r="H36" s="29"/>
@@ -2188,7 +2246,7 @@
         <x:v>I35</x:v>
       </x:c>
       <x:c r="B37" s="39" t="str">
-        <x:v>S05 공격 시험·원인 분석</x:v>
+        <x:v>S05 공격 재현·원인 분석</x:v>
       </x:c>
       <x:c r="C37" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -2196,7 +2254,9 @@
       <x:c r="D37" s="40" t="str">
         <x:v>11/02</x:v>
       </x:c>
-      <x:c r="E37" s="41" t="str"/>
+      <x:c r="E37" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F37" s="29"/>
       <x:c r="G37" s="29"/>
       <x:c r="H37" s="29"/>
@@ -2240,7 +2300,9 @@
       <x:c r="D38" s="23" t="str">
         <x:v>11/03</x:v>
       </x:c>
-      <x:c r="E38" s="24" t="str"/>
+      <x:c r="E38" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F38" s="29"/>
       <x:c r="G38" s="29"/>
       <x:c r="H38" s="29"/>
@@ -2276,7 +2338,7 @@
         <x:v>I16.1</x:v>
       </x:c>
       <x:c r="B39" s="39" t="str">
-        <x:v>M1 TO-BE 도면·정책 설계</x:v>
+        <x:v>M1 TO-BE 토폴로지·보안 정책 설계</x:v>
       </x:c>
       <x:c r="C39" s="40" t="str">
         <x:v>M1 유용수</x:v>
@@ -2284,7 +2346,9 @@
       <x:c r="D39" s="40" t="str">
         <x:v>11/03</x:v>
       </x:c>
-      <x:c r="E39" s="41" t="str"/>
+      <x:c r="E39" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F39" s="29"/>
       <x:c r="G39" s="29"/>
       <x:c r="H39" s="29"/>
@@ -2320,7 +2384,7 @@
         <x:v>I21.1</x:v>
       </x:c>
       <x:c r="B40" s="22" t="str">
-        <x:v>M2 TO-BE 도면·정책 설계</x:v>
+        <x:v>M2 TO-BE 토폴로지·보안 정책 설계</x:v>
       </x:c>
       <x:c r="C40" s="23" t="str">
         <x:v>M2 윤서영</x:v>
@@ -2328,7 +2392,9 @@
       <x:c r="D40" s="23" t="str">
         <x:v>11/03</x:v>
       </x:c>
-      <x:c r="E40" s="24" t="str"/>
+      <x:c r="E40" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F40" s="29"/>
       <x:c r="G40" s="29"/>
       <x:c r="H40" s="29"/>
@@ -2364,7 +2430,7 @@
         <x:v>I26.1</x:v>
       </x:c>
       <x:c r="B41" s="39" t="str">
-        <x:v>M3 TO-BE 도면·정책 설계</x:v>
+        <x:v>M3 TO-BE 토폴로지·보안 정책 설계</x:v>
       </x:c>
       <x:c r="C41" s="40" t="str">
         <x:v>M3 홍은서</x:v>
@@ -2372,7 +2438,9 @@
       <x:c r="D41" s="40" t="str">
         <x:v>11/03</x:v>
       </x:c>
-      <x:c r="E41" s="41" t="str"/>
+      <x:c r="E41" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F41" s="29"/>
       <x:c r="G41" s="29"/>
       <x:c r="H41" s="29"/>
@@ -2408,7 +2476,7 @@
         <x:v>I31.1</x:v>
       </x:c>
       <x:c r="B42" s="22" t="str">
-        <x:v>M4 TO-BE 도면·정책 설계</x:v>
+        <x:v>M4 TO-BE 토폴로지·보안 정책 설계</x:v>
       </x:c>
       <x:c r="C42" s="23" t="str">
         <x:v>M4 박진혁</x:v>
@@ -2416,7 +2484,9 @@
       <x:c r="D42" s="23" t="str">
         <x:v>11/03</x:v>
       </x:c>
-      <x:c r="E42" s="24" t="str"/>
+      <x:c r="E42" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F42" s="29"/>
       <x:c r="G42" s="29"/>
       <x:c r="H42" s="29"/>
@@ -2452,7 +2522,7 @@
         <x:v>I36.1</x:v>
       </x:c>
       <x:c r="B43" s="39" t="str">
-        <x:v>M5 TO-BE 도면·정책 설계</x:v>
+        <x:v>M5 TO-BE 토폴로지·보안 정책 설계</x:v>
       </x:c>
       <x:c r="C43" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -2460,7 +2530,9 @@
       <x:c r="D43" s="40" t="str">
         <x:v>11/03</x:v>
       </x:c>
-      <x:c r="E43" s="41" t="str"/>
+      <x:c r="E43" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F43" s="29"/>
       <x:c r="G43" s="29"/>
       <x:c r="H43" s="29"/>
@@ -2496,7 +2568,7 @@
         <x:v>MX1</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>M1 후속 실장비 간소화 설계</x:v>
+        <x:v>M1 후속 실장비 네트워크 설계</x:v>
       </x:c>
       <x:c r="C44" s="23" t="str">
         <x:v>M2 윤서영</x:v>
@@ -2504,7 +2576,9 @@
       <x:c r="D44" s="23" t="str">
         <x:v>미정</x:v>
       </x:c>
-      <x:c r="E44" s="24" t="str"/>
+      <x:c r="E44" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F44" s="29"/>
       <x:c r="G44" s="29"/>
       <x:c r="H44" s="29"/>
@@ -2537,7 +2611,7 @@
     </x:row>
     <x:row r="45" ht="21" customHeight="1">
       <x:c r="A45" s="42" t="str">
-        <x:v>기준: 원본 WBS 조회 2026.10.21 10:51 KST  |  원본 상태 “미확인”은 빈칸, 완료 2건은 E열 표시  |  MX1의 마감은 미정</x:v>
+        <x:v>2026.10.22 개정 | 등록·PL 기술 검토 구분 | M1–M3 일반 라우팅 결정 | 날짜는 목표·MX1 미정</x:v>
       </x:c>
       <x:c r="B45" s="42"/>
       <x:c r="C45" s="42"/>
@@ -2712,7 +2786,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>계획 기간은 옅은 칸으로 표시. 실제 진행한 날짜 칸을 색칠하고, 완료 확인 후 E열도 색칠하세요. 날짜 변경은 원본 WBS에 반영.</x:v>
+        <x:v>목표 기간은 옅은 칸. 수행일은 직접 색칠. 완료는 해당 작업 범위 기준이며 기술 검토와 구분합니다.</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -2808,7 +2882,7 @@
         <x:v>마감</x:v>
       </x:c>
       <x:c r="E5" s="14" t="str">
-        <x:v>완료</x:v>
+        <x:v>상태</x:v>
       </x:c>
       <x:c r="F5" s="14" t="str">
         <x:v>19</x:v>
@@ -2903,7 +2977,7 @@
         <x:v>D6.2</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>한국 CD·AI 공동 배포</x:v>
+        <x:v>한국 CD 구성·AI 서비스 배포</x:v>
       </x:c>
       <x:c r="C6" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -2911,7 +2985,9 @@
       <x:c r="D6" s="23" t="str">
         <x:v>11/04</x:v>
       </x:c>
-      <x:c r="E6" s="24" t="str"/>
+      <x:c r="E6" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F6" s="29"/>
       <x:c r="G6" s="29"/>
       <x:c r="H6" s="29"/>
@@ -2947,7 +3023,7 @@
         <x:v>D7</x:v>
       </x:c>
       <x:c r="B7" s="39" t="str">
-        <x:v>AI 실제 자막·웹 연동</x:v>
+        <x:v>AI 자막 생성·플레이어 기능 구현</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -2955,7 +3031,9 @@
       <x:c r="D7" s="40" t="str">
         <x:v>11/04</x:v>
       </x:c>
-      <x:c r="E7" s="41" t="str"/>
+      <x:c r="E7" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F7" s="29"/>
       <x:c r="G7" s="29"/>
       <x:c r="H7" s="29"/>
@@ -2991,7 +3069,7 @@
         <x:v>I26.2</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>S03·S05 정책·앱 분산 적용</x:v>
+        <x:v>S03·S05 접근제어·앱 부하 분산 적용</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
         <x:v>M3 홍은서</x:v>
@@ -2999,7 +3077,9 @@
       <x:c r="D8" s="23" t="str">
         <x:v>11/04</x:v>
       </x:c>
-      <x:c r="E8" s="24" t="str"/>
+      <x:c r="E8" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F8" s="29"/>
       <x:c r="G8" s="29"/>
       <x:c r="H8" s="29"/>
@@ -3035,7 +3115,7 @@
         <x:v>I31.2</x:v>
       </x:c>
       <x:c r="B9" s="39" t="str">
-        <x:v>백업 파일 권한·감사 적용</x:v>
+        <x:v>백업 파일 접근권한·감사 로그 설정</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
         <x:v>M4 박진혁</x:v>
@@ -3043,7 +3123,9 @@
       <x:c r="D9" s="40" t="str">
         <x:v>11/04</x:v>
       </x:c>
-      <x:c r="E9" s="41" t="str"/>
+      <x:c r="E9" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F9" s="29"/>
       <x:c r="G9" s="29"/>
       <x:c r="H9" s="29"/>
@@ -3079,7 +3161,7 @@
         <x:v>C10.3</x:v>
       </x:c>
       <x:c r="B10" s="22" t="str">
-        <x:v>별도 DB 첫 복원</x:v>
+        <x:v>격리 DB 초기 복원 테스트</x:v>
       </x:c>
       <x:c r="C10" s="23" t="str">
         <x:v>M4 박진혁</x:v>
@@ -3087,7 +3169,9 @@
       <x:c r="D10" s="23" t="str">
         <x:v>11/04</x:v>
       </x:c>
-      <x:c r="E10" s="24" t="str"/>
+      <x:c r="E10" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F10" s="29"/>
       <x:c r="G10" s="29"/>
       <x:c r="H10" s="29"/>
@@ -3123,7 +3207,7 @@
         <x:v>D6.3</x:v>
       </x:c>
       <x:c r="B11" s="39" t="str">
-        <x:v>Store CD 배포</x:v>
+        <x:v>Store CD 구성·자동 배포</x:v>
       </x:c>
       <x:c r="C11" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -3131,7 +3215,9 @@
       <x:c r="D11" s="40" t="str">
         <x:v>11/05</x:v>
       </x:c>
-      <x:c r="E11" s="41" t="str"/>
+      <x:c r="E11" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F11" s="29"/>
       <x:c r="G11" s="29"/>
       <x:c r="H11" s="29"/>
@@ -3167,7 +3253,7 @@
         <x:v>I16.2</x:v>
       </x:c>
       <x:c r="B12" s="22" t="str">
-        <x:v>직원 SSH 차단·관리 허용</x:v>
+        <x:v>직원망 SSH 차단·관리망 접근 허용</x:v>
       </x:c>
       <x:c r="C12" s="23" t="str">
         <x:v>M1 유용수</x:v>
@@ -3175,7 +3261,9 @@
       <x:c r="D12" s="23" t="str">
         <x:v>11/05</x:v>
       </x:c>
-      <x:c r="E12" s="24" t="str"/>
+      <x:c r="E12" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F12" s="29"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
@@ -3211,7 +3299,7 @@
         <x:v>I21.2</x:v>
       </x:c>
       <x:c r="B13" s="39" t="str">
-        <x:v>독일 Wazuh·대응 적용</x:v>
+        <x:v>독일 Wazuh 구축·대응 정책 적용</x:v>
       </x:c>
       <x:c r="C13" s="40" t="str">
         <x:v>M2 윤서영</x:v>
@@ -3219,7 +3307,9 @@
       <x:c r="D13" s="40" t="str">
         <x:v>11/05</x:v>
       </x:c>
-      <x:c r="E13" s="41" t="str"/>
+      <x:c r="E13" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F13" s="29"/>
       <x:c r="G13" s="29"/>
       <x:c r="H13" s="29"/>
@@ -3263,7 +3353,9 @@
       <x:c r="D14" s="23" t="str">
         <x:v>11/05</x:v>
       </x:c>
-      <x:c r="E14" s="24" t="str"/>
+      <x:c r="E14" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F14" s="29"/>
       <x:c r="G14" s="29"/>
       <x:c r="H14" s="29"/>
@@ -3299,7 +3391,7 @@
         <x:v>I31.3</x:v>
       </x:c>
       <x:c r="B15" s="39" t="str">
-        <x:v>원본 DB·Replica 첫 복제</x:v>
+        <x:v>원본·복제 DB 초기 동기화</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
         <x:v>M4 박진혁</x:v>
@@ -3307,7 +3399,9 @@
       <x:c r="D15" s="40" t="str">
         <x:v>11/05</x:v>
       </x:c>
-      <x:c r="E15" s="41" t="str"/>
+      <x:c r="E15" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F15" s="29"/>
       <x:c r="G15" s="29"/>
       <x:c r="H15" s="29"/>
@@ -3343,7 +3437,7 @@
         <x:v>C8</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>앱·AI·CI/CD 통합 확인</x:v>
+        <x:v>앱·AI·CI/CD 통합 테스트</x:v>
       </x:c>
       <x:c r="C16" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -3351,7 +3445,9 @@
       <x:c r="D16" s="23" t="str">
         <x:v>11/06</x:v>
       </x:c>
-      <x:c r="E16" s="24" t="str"/>
+      <x:c r="E16" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F16" s="29"/>
       <x:c r="G16" s="29"/>
       <x:c r="H16" s="29"/>
@@ -3387,7 +3483,7 @@
         <x:v>C10.4</x:v>
       </x:c>
       <x:c r="B17" s="39" t="str">
-        <x:v>S3 사본·격리 복원 확인</x:v>
+        <x:v>S3 백업본·격리 복원 검증</x:v>
       </x:c>
       <x:c r="C17" s="40" t="str">
         <x:v>M4 박진혁</x:v>
@@ -3395,7 +3491,9 @@
       <x:c r="D17" s="40" t="str">
         <x:v>11/06</x:v>
       </x:c>
-      <x:c r="E17" s="41" t="str"/>
+      <x:c r="E17" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F17" s="29"/>
       <x:c r="G17" s="29"/>
       <x:c r="H17" s="29"/>
@@ -3431,7 +3529,7 @@
         <x:v>I16.3</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>M1 개선 통합·정상 업무</x:v>
+        <x:v>M1 개선 설정 통합·정상 통신 검증</x:v>
       </x:c>
       <x:c r="C18" s="23" t="str">
         <x:v>M1 유용수</x:v>
@@ -3439,7 +3537,9 @@
       <x:c r="D18" s="23" t="str">
         <x:v>11/06</x:v>
       </x:c>
-      <x:c r="E18" s="24" t="str"/>
+      <x:c r="E18" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F18" s="29"/>
       <x:c r="G18" s="29"/>
       <x:c r="H18" s="29"/>
@@ -3475,7 +3575,7 @@
         <x:v>I21.3</x:v>
       </x:c>
       <x:c r="B19" s="39" t="str">
-        <x:v>독일 탐지·해제·업무 확인</x:v>
+        <x:v>독일 탐지·차단 해제·정상 동작 검증</x:v>
       </x:c>
       <x:c r="C19" s="40" t="str">
         <x:v>M2 윤서영</x:v>
@@ -3483,7 +3583,9 @@
       <x:c r="D19" s="40" t="str">
         <x:v>11/06</x:v>
       </x:c>
-      <x:c r="E19" s="41" t="str"/>
+      <x:c r="E19" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F19" s="29"/>
       <x:c r="G19" s="29"/>
       <x:c r="H19" s="29"/>
@@ -3519,7 +3621,7 @@
         <x:v>I26.4</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>M3 개선 구성 통합 확인</x:v>
+        <x:v>M3 개선 설정 통합 검증</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
         <x:v>M3 홍은서</x:v>
@@ -3527,7 +3629,9 @@
       <x:c r="D20" s="23" t="str">
         <x:v>11/06</x:v>
       </x:c>
-      <x:c r="E20" s="24" t="str"/>
+      <x:c r="E20" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F20" s="29"/>
       <x:c r="G20" s="29"/>
       <x:c r="H20" s="29"/>
@@ -3563,7 +3667,7 @@
         <x:v>I36.2</x:v>
       </x:c>
       <x:c r="B21" s="39" t="str">
-        <x:v>S05 정책·캐나다 경로 확인</x:v>
+        <x:v>S05 접근제어·캐나다 통신 경로 검증</x:v>
       </x:c>
       <x:c r="C21" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -3571,7 +3675,9 @@
       <x:c r="D21" s="40" t="str">
         <x:v>11/06</x:v>
       </x:c>
-      <x:c r="E21" s="41" t="str"/>
+      <x:c r="E21" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F21" s="29"/>
       <x:c r="G21" s="29"/>
       <x:c r="H21" s="29"/>
@@ -3607,7 +3713,7 @@
         <x:v>D8</x:v>
       </x:c>
       <x:c r="B22" s="22" t="str">
-        <x:v>앱 회귀·배포 버전 롤백</x:v>
+        <x:v>앱 회귀 테스트·배포 롤백 검증</x:v>
       </x:c>
       <x:c r="C22" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -3615,7 +3721,9 @@
       <x:c r="D22" s="23" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E22" s="24" t="str"/>
+      <x:c r="E22" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F22" s="29"/>
       <x:c r="G22" s="29"/>
       <x:c r="H22" s="29"/>
@@ -3651,7 +3759,7 @@
         <x:v>I17</x:v>
       </x:c>
       <x:c r="B23" s="39" t="str">
-        <x:v>S01 재시험·정상 업무 검증</x:v>
+        <x:v>S01 재공격·정상 동작 검증</x:v>
       </x:c>
       <x:c r="C23" s="40" t="str">
         <x:v>M1 유용수</x:v>
@@ -3659,7 +3767,9 @@
       <x:c r="D23" s="40" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E23" s="41" t="str"/>
+      <x:c r="E23" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F23" s="29"/>
       <x:c r="G23" s="29"/>
       <x:c r="H23" s="29"/>
@@ -3695,7 +3805,7 @@
         <x:v>I22</x:v>
       </x:c>
       <x:c r="B24" s="22" t="str">
-        <x:v>S02 재시험·정상 업무 검증</x:v>
+        <x:v>S02 재공격·정상 동작 검증</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
         <x:v>M2 윤서영</x:v>
@@ -3703,7 +3813,9 @@
       <x:c r="D24" s="23" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E24" s="24" t="str"/>
+      <x:c r="E24" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F24" s="29"/>
       <x:c r="G24" s="29"/>
       <x:c r="H24" s="29"/>
@@ -3739,7 +3851,7 @@
         <x:v>I27</x:v>
       </x:c>
       <x:c r="B25" s="39" t="str">
-        <x:v>S03 재시험·정상 업무 검증</x:v>
+        <x:v>S03 재공격·정상 동작 검증</x:v>
       </x:c>
       <x:c r="C25" s="40" t="str">
         <x:v>M3 홍은서</x:v>
@@ -3747,7 +3859,9 @@
       <x:c r="D25" s="40" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E25" s="41" t="str"/>
+      <x:c r="E25" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F25" s="29"/>
       <x:c r="G25" s="29"/>
       <x:c r="H25" s="29"/>
@@ -3783,7 +3897,7 @@
         <x:v>I32</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>S04 재시험·정상 업무 검증</x:v>
+        <x:v>S04 재공격·정상 동작 검증</x:v>
       </x:c>
       <x:c r="C26" s="23" t="str">
         <x:v>M4 박진혁</x:v>
@@ -3791,7 +3905,9 @@
       <x:c r="D26" s="23" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E26" s="24" t="str"/>
+      <x:c r="E26" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F26" s="29"/>
       <x:c r="G26" s="29"/>
       <x:c r="H26" s="29"/>
@@ -3827,7 +3943,7 @@
         <x:v>I37</x:v>
       </x:c>
       <x:c r="B27" s="39" t="str">
-        <x:v>S05 재시험·정상 업무 검증</x:v>
+        <x:v>S05 재공격·정상 동작 검증</x:v>
       </x:c>
       <x:c r="C27" s="40" t="str">
         <x:v>M5 유은혜</x:v>
@@ -3835,7 +3951,9 @@
       <x:c r="D27" s="40" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E27" s="41" t="str"/>
+      <x:c r="E27" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F27" s="29"/>
       <x:c r="G27" s="29"/>
       <x:c r="H27" s="29"/>
@@ -3879,7 +3997,9 @@
       <x:c r="D28" s="23" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E28" s="24" t="str"/>
+      <x:c r="E28" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F28" s="29"/>
       <x:c r="G28" s="29"/>
       <x:c r="H28" s="29"/>
@@ -3915,7 +4035,7 @@
         <x:v>C11.2</x:v>
       </x:c>
       <x:c r="B29" s="39" t="str">
-        <x:v>앱·노드·VIP 장애·복구 시험</x:v>
+        <x:v>앱·노드·VIP 장애 복구 테스트</x:v>
       </x:c>
       <x:c r="C29" s="40" t="str">
         <x:v>M3 홍은서</x:v>
@@ -3923,7 +4043,9 @@
       <x:c r="D29" s="40" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E29" s="41" t="str"/>
+      <x:c r="E29" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F29" s="29"/>
       <x:c r="G29" s="29"/>
       <x:c r="H29" s="29"/>
@@ -3959,7 +4081,7 @@
         <x:v>C12.3</x:v>
       </x:c>
       <x:c r="B30" s="22" t="str">
-        <x:v>RDS 별도 복원·자원 정리</x:v>
+        <x:v>RDS 격리 복원 검증·임시 자원 정리</x:v>
       </x:c>
       <x:c r="C30" s="23" t="str">
         <x:v>M5 유은혜</x:v>
@@ -3967,7 +4089,9 @@
       <x:c r="D30" s="23" t="str">
         <x:v>11/10</x:v>
       </x:c>
-      <x:c r="E30" s="24" t="str"/>
+      <x:c r="E30" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F30" s="29"/>
       <x:c r="G30" s="29"/>
       <x:c r="H30" s="29"/>
@@ -4011,7 +4135,9 @@
       <x:c r="D31" s="40" t="str">
         <x:v>11/12</x:v>
       </x:c>
-      <x:c r="E31" s="41" t="str"/>
+      <x:c r="E31" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F31" s="29"/>
       <x:c r="G31" s="29"/>
       <x:c r="H31" s="29"/>
@@ -4055,7 +4181,9 @@
       <x:c r="D32" s="23" t="str">
         <x:v>11/12</x:v>
       </x:c>
-      <x:c r="E32" s="24" t="str"/>
+      <x:c r="E32" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F32" s="29"/>
       <x:c r="G32" s="29"/>
       <x:c r="H32" s="29"/>
@@ -4099,7 +4227,9 @@
       <x:c r="D33" s="40" t="str">
         <x:v>11/12</x:v>
       </x:c>
-      <x:c r="E33" s="41" t="str"/>
+      <x:c r="E33" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F33" s="29"/>
       <x:c r="G33" s="29"/>
       <x:c r="H33" s="29"/>
@@ -4143,7 +4273,9 @@
       <x:c r="D34" s="23" t="str">
         <x:v>11/12</x:v>
       </x:c>
-      <x:c r="E34" s="24" t="str"/>
+      <x:c r="E34" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F34" s="29"/>
       <x:c r="G34" s="29"/>
       <x:c r="H34" s="29"/>
@@ -4187,7 +4319,9 @@
       <x:c r="D35" s="40" t="str">
         <x:v>11/12</x:v>
       </x:c>
-      <x:c r="E35" s="41" t="str"/>
+      <x:c r="E35" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F35" s="29"/>
       <x:c r="G35" s="29"/>
       <x:c r="H35" s="29"/>
@@ -4231,7 +4365,9 @@
       <x:c r="D36" s="23" t="str">
         <x:v>11/12</x:v>
       </x:c>
-      <x:c r="E36" s="24" t="str"/>
+      <x:c r="E36" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F36" s="29"/>
       <x:c r="G36" s="29"/>
       <x:c r="H36" s="29"/>
@@ -4275,7 +4411,9 @@
       <x:c r="D37" s="40" t="str">
         <x:v>11/13</x:v>
       </x:c>
-      <x:c r="E37" s="41" t="str"/>
+      <x:c r="E37" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F37" s="29"/>
       <x:c r="G37" s="29"/>
       <x:c r="H37" s="29"/>
@@ -4319,7 +4457,9 @@
       <x:c r="D38" s="23" t="str">
         <x:v>11/14</x:v>
       </x:c>
-      <x:c r="E38" s="24" t="str"/>
+      <x:c r="E38" s="24" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F38" s="29"/>
       <x:c r="G38" s="29"/>
       <x:c r="H38" s="29"/>
@@ -4363,7 +4503,9 @@
       <x:c r="D39" s="40" t="str">
         <x:v>11/16</x:v>
       </x:c>
-      <x:c r="E39" s="41" t="str"/>
+      <x:c r="E39" s="41" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="F39" s="29"/>
       <x:c r="G39" s="29"/>
       <x:c r="H39" s="29"/>
@@ -4396,7 +4538,7 @@
     </x:row>
     <x:row r="40" ht="21" customHeight="1">
       <x:c r="A40" s="42" t="str">
-        <x:v>기준: 원본 WBS 조회 2026.10.21 10:51 KST  |  원본 상태 “미확인”은 빈칸, 완료 2건은 E열 표시  |  MX1의 마감은 미정</x:v>
+        <x:v>2026.10.22 개정 | 등록·PL 기술 검토 구분 | M1–M3 일반 라우팅 결정 | 날짜는 목표·MX1 미정</x:v>
       </x:c>
       <x:c r="B40" s="42"/>
       <x:c r="C40" s="42"/>

</xml_diff>